<commit_message>
Making price increase changes
</commit_message>
<xml_diff>
--- a/Interim Analyses/average_retail_summary_prices.xlsx
+++ b/Interim Analyses/average_retail_summary_prices.xlsx
@@ -402,10 +402,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>37.37264228177808</v>
+        <v>50.58672988860226</v>
       </c>
       <c r="D3">
-        <v>373.7264228177808</v>
+        <v>505.8672988860226</v>
       </c>
     </row>
     <row r="4">
@@ -434,10 +434,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>36.99624456155861</v>
+        <v>50.63799720292315</v>
       </c>
       <c r="D5">
-        <v>369.9624456155861</v>
+        <v>506.3799720292316</v>
       </c>
     </row>
     <row r="6">
@@ -466,10 +466,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>37.40998685408257</v>
+        <v>51.19499738525468</v>
       </c>
       <c r="D7">
-        <v>374.0998685408256</v>
+        <v>511.9499738525468</v>
       </c>
     </row>
     <row r="8">
@@ -498,10 +498,10 @@
         </is>
       </c>
       <c r="C9">
-        <v>36.25752547375507</v>
+        <v>48.42279383485617</v>
       </c>
       <c r="D9">
-        <v>362.5752547375507</v>
+        <v>484.2279383485616</v>
       </c>
     </row>
     <row r="10">
@@ -530,10 +530,10 @@
         </is>
       </c>
       <c r="C11">
-        <v>34.10979864276023</v>
+        <v>43.62797066175398</v>
       </c>
       <c r="D11">
-        <v>341.0979864276023</v>
+        <v>436.2797066175398</v>
       </c>
     </row>
     <row r="12">
@@ -562,10 +562,10 @@
         </is>
       </c>
       <c r="C13">
-        <v>32.37118176493082</v>
+        <v>39.85678589225297</v>
       </c>
       <c r="D13">
-        <v>323.7118176493082</v>
+        <v>398.5678589225297</v>
       </c>
     </row>
     <row r="14">
@@ -594,10 +594,10 @@
         </is>
       </c>
       <c r="C15">
-        <v>29.89080854652495</v>
+        <v>37.11483730157239</v>
       </c>
       <c r="D15">
-        <v>298.9080854652495</v>
+        <v>371.148373015724</v>
       </c>
     </row>
     <row r="16">
@@ -626,10 +626,10 @@
         </is>
       </c>
       <c r="C17">
-        <v>36.85201302697126</v>
+        <v>50.78380646606977</v>
       </c>
       <c r="D17">
-        <v>368.5201302697126</v>
+        <v>507.8380646606977</v>
       </c>
     </row>
     <row r="18">
@@ -658,10 +658,10 @@
         </is>
       </c>
       <c r="C19">
-        <v>38.92983287378097</v>
+        <v>54.93909578100293</v>
       </c>
       <c r="D19">
-        <v>389.2983287378098</v>
+        <v>549.3909578100294</v>
       </c>
     </row>
     <row r="20">
@@ -690,10 +690,10 @@
         </is>
       </c>
       <c r="C21">
-        <v>38.25719892346471</v>
+        <v>53.24963453051074</v>
       </c>
       <c r="D21">
-        <v>382.5719892346471</v>
+        <v>532.4963453051074</v>
       </c>
     </row>
     <row r="22">
@@ -722,10 +722,10 @@
         </is>
       </c>
       <c r="C23">
-        <v>39.40608906474425</v>
+        <v>55.34508667708951</v>
       </c>
       <c r="D23">
-        <v>394.0608906474425</v>
+        <v>553.4508667708951</v>
       </c>
     </row>
     <row r="24">
@@ -754,10 +754,10 @@
         </is>
       </c>
       <c r="C25">
-        <v>39.01451516751724</v>
+        <v>54.32068743153667</v>
       </c>
       <c r="D25">
-        <v>390.1451516751724</v>
+        <v>543.2068743153667</v>
       </c>
     </row>
     <row r="26">
@@ -786,10 +786,10 @@
         </is>
       </c>
       <c r="C27">
-        <v>37.6691197302488</v>
+        <v>51.82057125068759</v>
       </c>
       <c r="D27">
-        <v>376.691197302488</v>
+        <v>518.2057125068759</v>
       </c>
     </row>
     <row r="28">
@@ -818,10 +818,10 @@
         </is>
       </c>
       <c r="C29">
-        <v>39.27226073946576</v>
+        <v>55.00492415997298</v>
       </c>
       <c r="D29">
-        <v>392.7226073946576</v>
+        <v>550.0492415997298</v>
       </c>
     </row>
     <row r="30">
@@ -850,10 +850,10 @@
         </is>
       </c>
       <c r="C31">
-        <v>37.64395405889712</v>
+        <v>51.82337881367276</v>
       </c>
       <c r="D31">
-        <v>376.4395405889712</v>
+        <v>518.2337881367276</v>
       </c>
     </row>
     <row r="32">
@@ -882,10 +882,10 @@
         </is>
       </c>
       <c r="C33">
-        <v>37.61521532391023</v>
+        <v>51.84922564032955</v>
       </c>
       <c r="D33">
-        <v>376.1521532391023</v>
+        <v>518.4922564032955</v>
       </c>
     </row>
     <row r="34">
@@ -914,10 +914,10 @@
         </is>
       </c>
       <c r="C35">
-        <v>37.50612520031127</v>
+        <v>51.67790911388461</v>
       </c>
       <c r="D35">
-        <v>375.0612520031127</v>
+        <v>516.7790911388461</v>
       </c>
     </row>
     <row r="36">
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="C37">
-        <v>37.75041328815276</v>
+        <v>52.20851506459212</v>
       </c>
       <c r="D37">
-        <v>377.5041328815275</v>
+        <v>522.0851506459212</v>
       </c>
     </row>
     <row r="38">
@@ -978,10 +978,10 @@
         </is>
       </c>
       <c r="C39">
-        <v>38.40710133568324</v>
+        <v>53.6246702857712</v>
       </c>
       <c r="D39">
-        <v>384.0710133568324</v>
+        <v>536.246702857712</v>
       </c>
     </row>
     <row r="40">
@@ -1010,10 +1010,10 @@
         </is>
       </c>
       <c r="C41">
-        <v>39.87730474929839</v>
+        <v>56.55742427641282</v>
       </c>
       <c r="D41">
-        <v>398.7730474929839</v>
+        <v>565.5742427641281</v>
       </c>
     </row>
     <row r="42">
@@ -1042,10 +1042,10 @@
         </is>
       </c>
       <c r="C43">
-        <v>41.40049524731685</v>
+        <v>59.55552169520107</v>
       </c>
       <c r="D43">
-        <v>414.0049524731685</v>
+        <v>595.5552169520107</v>
       </c>
     </row>
     <row r="44">
@@ -1074,10 +1074,10 @@
         </is>
       </c>
       <c r="C45">
-        <v>41.33937795361415</v>
+        <v>59.43002670749483</v>
       </c>
       <c r="D45">
-        <v>413.3937795361415</v>
+        <v>594.3002670749484</v>
       </c>
     </row>
     <row r="46">
@@ -1106,10 +1106,10 @@
         </is>
       </c>
       <c r="C47">
-        <v>40.26556933457412</v>
+        <v>57.30892701013831</v>
       </c>
       <c r="D47">
-        <v>402.6556933457413</v>
+        <v>573.089270101383</v>
       </c>
     </row>
     <row r="48">
@@ -1138,10 +1138,10 @@
         </is>
       </c>
       <c r="C49">
-        <v>39.9326179817832</v>
+        <v>56.67584484270009</v>
       </c>
       <c r="D49">
-        <v>399.326179817832</v>
+        <v>566.758448427001</v>
       </c>
     </row>
     <row r="50">
@@ -1170,10 +1170,10 @@
         </is>
       </c>
       <c r="C51">
-        <v>40.65631539060816</v>
+        <v>58.0796718239372</v>
       </c>
       <c r="D51">
-        <v>406.5631539060815</v>
+        <v>580.796718239372</v>
       </c>
     </row>
     <row r="52">
@@ -1202,10 +1202,10 @@
         </is>
       </c>
       <c r="C53">
-        <v>40.76012513985776</v>
+        <v>58.29784093261392</v>
       </c>
       <c r="D53">
-        <v>407.6012513985776</v>
+        <v>582.9784093261392</v>
       </c>
     </row>
   </sheetData>

</xml_diff>